<commit_message>
Updated pics and roster
</commit_message>
<xml_diff>
--- a/game-stats/Week4_Desert-Lions_vs_Darkside.xlsx
+++ b/game-stats/Week4_Desert-Lions_vs_Darkside.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S19"/>
+  <dimension ref="A1:S20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1772,6 +1772,69 @@
         <v>0</v>
       </c>
       <c r="S19" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Moe Ashkar</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>OL</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated week 4 schedule
</commit_message>
<xml_diff>
--- a/game-stats/Week4_Desert-Lions_vs_Darkside.xlsx
+++ b/game-stats/Week4_Desert-Lions_vs_Darkside.xlsx
@@ -535,13 +535,15 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
     <col width="11" customWidth="1" min="16" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1862,13 +1864,15 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
     <col width="11" customWidth="1" min="16" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>